<commit_message>
📦 Phase 1: Order Confirmation + Feedback Flow
- orderFlow.js: Full state machine (availability → confirm → deliver → feedback)
- adminRouter.js: Admin API endpoints
- webhook.js: Order flow intercepts messages before AI
- index.js: /admin routes mounted

Flow:
1. Deal close → 30s later: 'Busy ya free?' text
2. Customer: 'Free' → Order details + confirm request
3. Customer: 'Confirm' → Excel status = Confirmed
4. Admin: POST /admin/mark-delivered → Feedback request sent
5. Customer: Feedback → Saved to feedback.xlsx
</commit_message>
<xml_diff>
--- a/data/customers.xlsx
+++ b/data/customers.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -64,8 +65,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,131 +414,101 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" s="1" t="str">
+        <v>Amount</v>
+      </c>
+      <c r="B1" s="1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" s="1" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="D1" s="1" t="str">
+        <v>FollowUpDate</v>
+      </c>
+      <c r="E1" s="1" t="str">
+        <v>FollowUpDone</v>
+      </c>
+      <c r="F1" s="1" t="str">
         <v>Timestamp</v>
       </c>
-      <c r="B1" t="str">
+      <c r="G1" s="1" t="str">
         <v>Phone</v>
       </c>
-      <c r="C1" t="str">
+      <c r="H1" s="1" t="str">
         <v>Name</v>
       </c>
-      <c r="D1" t="str">
+      <c r="I1" s="1" t="str">
         <v>Address</v>
       </c>
-      <c r="E1" t="str">
+      <c r="J1" s="1" t="str">
         <v>Product</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Amount</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Notes</v>
-      </c>
-      <c r="I1" t="str">
-        <v>FollowUpDate</v>
-      </c>
-      <c r="J1" t="str">
-        <v>FollowUpDone</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>2026-05-08T13:43:05.671Z</v>
-      </c>
-      <c r="B2" t="str">
-        <v>923001234567</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Ahmed Bhai</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Lahore, DHA Phase 5</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Italian Wool Blazer</v>
-      </c>
-      <c r="F2">
-        <v>185</v>
-      </c>
-      <c r="G2" t="str">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="str">
         <v>New</v>
       </c>
-      <c r="H2" t="str">
-        <v>Test deal - confirm karo bola</v>
-      </c>
-      <c r="I2" t="str">
-        <v>2026-05-23</v>
-      </c>
-      <c r="J2" t="b">
+      <c r="C2" s="1" t="str">
+        <v>mai yh product ku buy kru kia warrenty hai yh sai hogi ?</v>
+      </c>
+      <c r="D2" s="1" t="str">
+        <v>2026-05-21</v>
+      </c>
+      <c r="E2" s="1" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>2026-05-08T13:44:09.724Z</v>
-      </c>
-      <c r="B3" t="str">
-        <v>923424747228</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Awais Sabir</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Islamabad</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Italian Wool Blazer</v>
-      </c>
-      <c r="F3">
+      <c r="A3" s="1">
         <v>0</v>
       </c>
-      <c r="G3" t="str">
+      <c r="B3" s="1" t="str">
         <v>New</v>
       </c>
-      <c r="H3" t="str">
-        <v>Name: Awais sabir , Address ;Islamabad , phone Number : 03424747228</v>
-      </c>
-      <c r="I3" t="str">
+      <c r="C3" s="1" t="str">
+        <v>chalo order confirm krty lkn mjy ap apni policy to btao</v>
+      </c>
+      <c r="D3" s="1" t="str">
         <v>2026-05-23</v>
       </c>
-      <c r="J3" t="b">
+      <c r="E3" s="1" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>2026-05-08T13:54:19.918Z</v>
-      </c>
-      <c r="B4" t="str">
+      <c r="A4" s="1">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>New</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>Name : Awais , Address: Islamabad , Number ; 03424747228</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="E4" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="str">
+        <v>2026-05-08T18:37:55.074Z</v>
+      </c>
+      <c r="G4" s="1" t="str">
         <v>923424747228</v>
       </c>
-      <c r="C4" t="str">
-        <v>Not provided</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Signature Oxford Shirt</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4" t="str">
-        <v>New</v>
-      </c>
-      <c r="H4" t="str">
-        <v>yes confirm kro order</v>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-05-18</v>
-      </c>
-      <c r="J4" t="b">
-        <v>0</v>
+      <c r="H4" s="1" t="str">
+        <v>Awais</v>
+      </c>
+      <c r="I4" s="1" t="str">
+        <v>Islamabad</v>
+      </c>
+      <c r="J4" s="1" t="str">
+        <v>Italian Wool Blazer</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🗑️ Removed Phase 1 order flow — back to simple AI chat
- Removed orderFlow intercept from webhook.js
- Removed adminRouter from index.js
- Agent now handles all messages directly via GPT-4o
- Deal logging still works (Excel + Supabase)
</commit_message>
<xml_diff>
--- a/data/customers.xlsx
+++ b/data/customers.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J6"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -511,9 +511,73 @@
         <v>Italian Wool Blazer</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>0</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>Confirmed</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>Islamabad address hai</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <v>2026-05-21</v>
+      </c>
+      <c r="E5" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="str">
+        <v>2026-05-08T20:39:41.311Z</v>
+      </c>
+      <c r="G5" s="1" t="str">
+        <v>923295049923</v>
+      </c>
+      <c r="H5" s="1" t="str">
+        <v>Saif</v>
+      </c>
+      <c r="I5" s="1" t="str">
+        <v>Islamabad</v>
+      </c>
+      <c r="J5" s="1" t="str">
+        <v>Modern Oxford Shoes</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>0</v>
+      </c>
+      <c r="B6" s="1" t="str">
+        <v>New</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <v>Order pe maira name kia likha tha, aur ab tak main Kitne order kar Chuka hoon</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <v>2026-05-19</v>
+      </c>
+      <c r="E6" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="str">
+        <v>2026-05-08T20:46:09.919Z</v>
+      </c>
+      <c r="G6" s="1" t="str">
+        <v>923295049923</v>
+      </c>
+      <c r="H6" s="1" t="str">
+        <v>Saif Iqbal</v>
+      </c>
+      <c r="I6" s="1" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="J6" s="1" t="str">
+        <v>Unknown</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
📍 Pakistani phone validation + Location map feature
Feature 1 - Phone Validation:
- AI validates 11-digit Pakistani numbers (03XX format)
- Rejects: 10 digits, country code format (923XX)
- Politely asks customer to re-enter if wrong

Feature 2 - Address Map:
- When customer gives address, AI triggers [ADDRESS_CONFIRMED]
- System geocodes address via Nominatim (free, no API key)
- Sends Google Maps link to customer for verification
- If GEOAPIFY_API_KEY set: sends static map image instead
- Customer confirms: 'Haan sahi hai' or corrects address

New files: src/mapHandler.js
</commit_message>
<xml_diff>
--- a/data/customers.xlsx
+++ b/data/customers.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J9"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -575,9 +575,105 @@
         <v>Unknown</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>0</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <v>New</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <v>Islamabad ,03424747228</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <v>2026-05-25</v>
+      </c>
+      <c r="E7" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="str">
+        <v>2026-05-10T11:30:49.341Z</v>
+      </c>
+      <c r="G7" s="1" t="str">
+        <v>923424747228</v>
+      </c>
+      <c r="H7" s="1" t="str">
+        <v>Awais</v>
+      </c>
+      <c r="I7" s="1" t="str">
+        <v>Islamabad</v>
+      </c>
+      <c r="J7" s="1" t="str">
+        <v>Signature Oxford Shirt</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>0</v>
+      </c>
+      <c r="B8" s="1" t="str">
+        <v>New</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <v>Ali, I 11, 12345678912</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <v>2026-05-21</v>
+      </c>
+      <c r="E8" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1" t="str">
+        <v>2026-05-10T11:52:40.964Z</v>
+      </c>
+      <c r="G8" s="1" t="str">
+        <v>923464800136</v>
+      </c>
+      <c r="H8" s="1" t="str">
+        <v>Ali</v>
+      </c>
+      <c r="I8" s="1" t="str">
+        <v>I 11</v>
+      </c>
+      <c r="J8" s="1" t="str">
+        <v>Italian Wool Blazer</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>0</v>
+      </c>
+      <c r="B9" s="1" t="str">
+        <v>New</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <v>Acha ap nai order confrm kesy kiya hain mainy ap ko Apna size hi nahi bataya or na Color</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <v>2026-05-21</v>
+      </c>
+      <c r="E9" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1" t="str">
+        <v>2026-05-10T11:53:26.221Z</v>
+      </c>
+      <c r="G9" s="1" t="str">
+        <v>923464800136</v>
+      </c>
+      <c r="H9" s="1" t="str">
+        <v>M..Asim</v>
+      </c>
+      <c r="I9" s="1" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="J9" s="1" t="str">
+        <v>Unknown</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
📍 Smart address collection — city vs village flow
- Step 1: AI asks 'City ya Village area?'
- City flow: House no + Street + Area + City (all required)
- Village flow: Nearest bazaar/landmark + Village + Tehsil + District
- Never confirms incomplete address — asks for missing fields
- Full address repeated to customer before [ADDRESS_CONFIRMED]
</commit_message>
<xml_diff>
--- a/data/customers.xlsx
+++ b/data/customers.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J11"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -671,9 +671,73 @@
         <v>Unknown</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>0</v>
+      </c>
+      <c r="B10" s="1" t="str">
+        <v>New</v>
+      </c>
+      <c r="C10" s="1" t="str">
+        <v>asim, Islamabd</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <v>2026-05-22</v>
+      </c>
+      <c r="E10" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1" t="str">
+        <v>2026-05-10T12:24:39.897Z</v>
+      </c>
+      <c r="G10" s="1" t="str">
+        <v>923464800136</v>
+      </c>
+      <c r="H10" s="1" t="str">
+        <v>Asim</v>
+      </c>
+      <c r="I10" s="1" t="str">
+        <v>Islamabad</v>
+      </c>
+      <c r="J10" s="1" t="str">
+        <v>Linen Summer Blazer</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>0</v>
+      </c>
+      <c r="B11" s="1" t="str">
+        <v>New</v>
+      </c>
+      <c r="C11" s="1" t="str">
+        <v>Islamabad</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <v>2026-05-21</v>
+      </c>
+      <c r="E11" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1" t="str">
+        <v>2026-05-10T12:25:54.022Z</v>
+      </c>
+      <c r="G11" s="1" t="str">
+        <v>923464800136</v>
+      </c>
+      <c r="H11" s="1" t="str">
+        <v>Asim</v>
+      </c>
+      <c r="I11" s="1" t="str">
+        <v>Islamabad</v>
+      </c>
+      <c r="J11" s="1" t="str">
+        <v>Linen Summer Blazer</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>